<commit_message>
adding unit 4 content
</commit_message>
<xml_diff>
--- a/unit3_databaseDesign/datasets/unit3e_Baseball.xlsx
+++ b/unit3_databaseDesign/datasets/unit3e_Baseball.xlsx
@@ -488,7 +488,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1. Open it in Google Sheets (File → Import → Upload). Share it with your partner so you both can edit.</t>
+          <t>1. Open it in Microsoft Excel. Save it in your repo as unit3e_Baseball_lastname.xlsx. Work on one copy with your partner.</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Select the bats_throws column, then Data → Split text to columns → Separator: Custom → type /</t>
+          <t xml:space="preserve">   Select the bats_throws column, then Data → Text to Columns → Delimited → Next → check Other and type / → Finish.</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Copy the columns you need from the 1NF tab, then use Data → Data cleanup → Remove duplicates.</t>
+          <t xml:space="preserve">   Copy the columns you need from the 1NF tab, then use Data → Remove Duplicates (check 'My data has headers').</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>7. When you finish, answer the questions in unit3e_Baseball_lastname.md and paste your table designs there.</t>
+          <t>7. When you finish, answer the questions in unit3e_Baseball_lastname.md and paste your table designs there. Commit this Excel file too.</t>
         </is>
       </c>
     </row>
@@ -26167,7 +26167,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Same data as Client_Export. Split the yellow bats_throws column into bats and throws (Data → Split text to columns, separator /).</t>
+          <t>Same data as Client_Export. Split the yellow bats_throws column into bats and throws (Data → Text to Columns → Delimited → Other: /).</t>
         </is>
       </c>
     </row>

</xml_diff>